<commit_message>
add details for report, add gitkeep handler, add gitignore
</commit_message>
<xml_diff>
--- a/template/template_semester.xlsx
+++ b/template/template_semester.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jafarfadli/Koding/SOTM/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CAB0EA7-9102-4F41-A772-E3F8701FCCD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5BB3E92-A70A-CC44-897B-DF16F80F3E15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="600" windowWidth="28800" windowHeight="15680" xr2:uid="{96D2B414-ED70-F542-80B9-37701F9EDC31}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15680" xr2:uid="{96D2B414-ED70-F542-80B9-37701F9EDC31}"/>
   </bookViews>
   <sheets>
     <sheet name="SUMMARY" sheetId="1" r:id="rId1"/>
+    <sheet name="DETAILS" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="14">
   <si>
     <t>SEMESTER</t>
   </si>
@@ -66,6 +67,18 @@
   </si>
   <si>
     <t>20XX</t>
+  </si>
+  <si>
+    <t>KODE MK</t>
+  </si>
+  <si>
+    <t>ETXXXX</t>
+  </si>
+  <si>
+    <t>NAMA MK</t>
+  </si>
+  <si>
+    <t>DOSEN</t>
   </si>
 </sst>
 </file>
@@ -169,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -198,6 +211,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2369,4 +2388,162 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31D3CE6B-3291-3847-9F27-C5CBE050149D}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="2"/>
+      <c r="B1" s="3"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="12"/>
+      <c r="B3" s="3"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="12"/>
+      <c r="B7" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="12"/>
+      <c r="B8" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="12"/>
+      <c r="B9" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="4">
+        <v>1</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="4">
+        <v>2</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="4">
+        <v>3</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="4">
+        <v>4</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="4">
+        <v>5</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="4">
+        <v>6</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="4">
+        <v>7</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="4">
+        <v>8</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="4">
+        <v>9</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="4">
+        <v>10</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>